<commit_message>
Planilha: linha do tablero da rede; registro dos slides de impacto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MG6VeavRZnDbjYZyzDjvL
</commit_message>
<xml_diff>
--- a/docs/negocio/SIVEC-metrica-SantaCruz.xlsx
+++ b/docs/negocio/SIVEC-metrica-SantaCruz.xlsx
@@ -160,6 +160,7 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,7 +182,6 @@
     <xf numFmtId="166" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,6 +195,7 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -204,7 +205,6 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="10" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -643,19 +643,19 @@
         </is>
       </c>
       <c r="B5" s="45">
-        <f>Estabelecimentos!D11</f>
+        <f>Estabelecimentos!D12</f>
         <v/>
       </c>
       <c r="C5" s="45">
-        <f>Estabelecimentos!E11</f>
+        <f>Estabelecimentos!E12</f>
         <v/>
       </c>
       <c r="D5" s="45">
-        <f>Estabelecimentos!E11</f>
+        <f>Estabelecimentos!E12</f>
         <v/>
       </c>
       <c r="E5" s="45">
-        <f>Estabelecimentos!F11</f>
+        <f>Estabelecimentos!F12</f>
         <v/>
       </c>
     </row>
@@ -666,19 +666,19 @@
         </is>
       </c>
       <c r="B6" s="46">
-        <f>Estabelecimentos!D12</f>
+        <f>Estabelecimentos!D13</f>
         <v/>
       </c>
       <c r="C6" s="46">
-        <f>Estabelecimentos!E12</f>
+        <f>Estabelecimentos!E13</f>
         <v/>
       </c>
       <c r="D6" s="46">
-        <f>Estabelecimentos!E12</f>
+        <f>Estabelecimentos!E13</f>
         <v/>
       </c>
       <c r="E6" s="46">
-        <f>Estabelecimentos!F12</f>
+        <f>Estabelecimentos!F13</f>
         <v/>
       </c>
     </row>
@@ -1011,19 +1011,19 @@
         </is>
       </c>
       <c r="B21" s="46">
-        <f>Estabelecimentos!D13</f>
+        <f>Estabelecimentos!D14</f>
         <v/>
       </c>
       <c r="C21" s="46">
-        <f>Estabelecimentos!E13</f>
+        <f>Estabelecimentos!E14</f>
         <v/>
       </c>
       <c r="D21" s="46">
-        <f>Estabelecimentos!E13</f>
+        <f>Estabelecimentos!E14</f>
         <v/>
       </c>
       <c r="E21" s="46">
-        <f>Estabelecimentos!F13</f>
+        <f>Estabelecimentos!F14</f>
         <v/>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -1350,6 +1350,36 @@
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Pagamento público costuma atrasar 60–90 dias: é o caixa que você precisa ter antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Mensalidade · tablero da rede e administração (US$)</t>
+        </is>
+      </c>
+      <c r="B17" s="56" t="n">
+        <v>250</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Como está no slide de preços. O slide "Incluye" diz que o tablero vem incluído: decidir qual vale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Implantação única · tablero da rede (US$)</t>
+        </is>
+      </c>
+      <c r="B18" s="56" t="n">
+        <v>250</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Como está no slide de preços.</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1441,13 +1471,13 @@
         <f>Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="D5" s="56" t="n">
+      <c r="D5" s="57" t="n">
         <v>8</v>
       </c>
-      <c r="E5" s="57" t="n">
+      <c r="E5" s="58" t="n">
         <v>60</v>
       </c>
-      <c r="F5" s="57" t="n">
+      <c r="F5" s="58" t="n">
         <v>160</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1470,13 +1500,13 @@
         <f>Supostos!$B$9</f>
         <v/>
       </c>
-      <c r="D6" s="56" t="n">
+      <c r="D6" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="57" t="n">
+      <c r="E6" s="58" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="57" t="n">
+      <c r="F6" s="58" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1499,13 +1529,13 @@
         <f>Supostos!$B$10</f>
         <v/>
       </c>
-      <c r="D7" s="56" t="n">
+      <c r="D7" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="56" t="n">
+      <c r="E7" s="57" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="57" t="n">
+      <c r="F7" s="58" t="n">
         <v>15</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1528,13 +1558,13 @@
         <f>Supostos!$B$11</f>
         <v/>
       </c>
-      <c r="D8" s="56" t="n">
+      <c r="D8" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="57" t="n">
+      <c r="E8" s="58" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="57" t="n">
+      <c r="F8" s="58" t="n">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1557,13 +1587,13 @@
         <f>Supostos!$B$11</f>
         <v/>
       </c>
-      <c r="D9" s="56" t="n">
+      <c r="D9" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="56" t="n">
+      <c r="E9" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="56" t="n">
+      <c r="F9" s="57" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1586,13 +1616,13 @@
         <f>Supostos!$B$11</f>
         <v/>
       </c>
-      <c r="D10" s="56" t="n">
+      <c r="D10" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="56" t="n">
+      <c r="E10" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="56" t="n">
+      <c r="F10" s="57" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1602,126 +1632,155 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Tablero da rede (gestor + mapa)</t>
+        </is>
+      </c>
+      <c r="B11" s="46">
+        <f>Supostos!$B$17</f>
+        <v/>
+      </c>
+      <c r="C11" s="46">
+        <f>Supostos!$B$18</f>
+        <v/>
+      </c>
+      <c r="D11" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Em 0 = incluído no pacote (como no exemplo da apresentação). Ponha 1 por rede se for cobrar os US$ 250 do slide de preços (Município: 4 redes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>TOTAL de estabelecimentos</t>
         </is>
       </c>
-      <c r="B11" s="25" t="n"/>
-      <c r="C11" s="25" t="n"/>
-      <c r="D11" s="58">
-        <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="58">
-        <f>SUM(E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="58">
-        <f>SUM(F5:F10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Mensalidades (US$/mês)</t>
-        </is>
-      </c>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="26" t="n"/>
       <c r="D12" s="59">
-        <f>SUMPRODUCT($B$5:$B$10,D5:D10)</f>
+        <f>SUM(D5:D11)</f>
         <v/>
       </c>
       <c r="E12" s="59">
-        <f>SUMPRODUCT($B$5:$B$10,E5:E10)</f>
+        <f>SUM(E5:E11)</f>
         <v/>
       </c>
       <c r="F12" s="59">
-        <f>SUMPRODUCT($B$5:$B$10,F5:F10)</f>
+        <f>SUM(F5:F11)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
+          <t>Mensalidades (US$/mês)</t>
+        </is>
+      </c>
+      <c r="D13" s="60">
+        <f>SUMPRODUCT($B$5:$B$11,D5:D11)</f>
+        <v/>
+      </c>
+      <c r="E13" s="60">
+        <f>SUMPRODUCT($B$5:$B$11,E5:E11)</f>
+        <v/>
+      </c>
+      <c r="F13" s="60">
+        <f>SUMPRODUCT($B$5:$B$11,F5:F11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>Implantação total (US$, uma vez)</t>
         </is>
       </c>
-      <c r="D13" s="59">
-        <f>SUMPRODUCT($C$5:$C$10,D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E13" s="59">
-        <f>SUMPRODUCT($C$5:$C$10,E5:E10)</f>
-        <v/>
-      </c>
-      <c r="F13" s="59">
-        <f>SUMPRODUCT($C$5:$C$10,F5:F10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="D14" s="60">
+        <f>SUMPRODUCT($C$5:$C$11,D5:D11)</f>
+        <v/>
+      </c>
+      <c r="E14" s="60">
+        <f>SUMPRODUCT($C$5:$C$11,E5:E11)</f>
+        <v/>
+      </c>
+      <c r="F14" s="60">
+        <f>SUMPRODUCT($C$5:$C$11,F5:F11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Lista de referência · município de Santa Cruz de la Sierra</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>4 redes municipais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Red Centro, Red Norte, Red Sur, Red Este (GAM Santa Cruz). O tablero da rede vem incluído no pacote.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Red Centro · 9 centros</t>
+          <t>4 redes municipais</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Elvira Wunderlich, Perpetuo Socorro, Roque Aguilera, San Carlos, San Luis, Santa Rosita, Virgen de Cotoca, Virgen de Fátima, Willy Lemaitre.</t>
+          <t>Red Centro, Red Norte, Red Sur, Red Este (GAM Santa Cruz). Tablero da rede: ver a linha "Tablero da rede" acima.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Hospitais municipais de 2º nível</t>
+          <t>Red Centro · 9 centros</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Francés, Villa 1ro de Mayo, Pampa de la Isla, Plan 3000, Bajío del Oriente.</t>
+          <t>Elvira Wunderlich, Perpetuo Socorro, Roque Aguilera, San Carlos, San Luis, Santa Rosita, Virgen de Cotoca, Virgen de Fátima, Willy Lemaitre.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Hospitais de 3º nível</t>
+          <t>Hospitais municipais de 2º nível</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>San Juan de Dios, Japonés, de Niños Dr. Mario Ortiz Suárez, de la Mujer Dr. Percy Boland, 5º a confirmar.</t>
+          <t>Francés, Villa 1ro de Mayo, Pampa de la Isla, Plan 3000, Bajío del Oriente.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
+          <t>Hospitais de 3º nível</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>San Juan de Dios, Japonés, de Niños Dr. Mario Ortiz Suárez, de la Mujer Dr. Percy Boland, 5º a confirmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
           <t>4º nível</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Instituto Oncológico del Oriente Boliviano.</t>
         </is>
@@ -1837,27 +1896,27 @@
           <t>Fundador / diretor</t>
         </is>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>Você: produto, parte clínica, contratos com o município e o SEDES. Na Red Centro você segue como médico e não tira salário.</t>
         </is>
       </c>
-      <c r="C5" s="60" t="n">
+      <c r="C5" s="61" t="n">
         <v>10000</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="56" t="n">
+      <c r="E5" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="56" t="n">
+      <c r="F5" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="56" t="n">
+      <c r="G5" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="56" t="n">
+      <c r="H5" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I5" s="48">
@@ -1883,27 +1942,27 @@
           <t>Desenvolvedor full-stack</t>
         </is>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Correções, melhorias, relatórios novos; responde pelo sistema perante o município.</t>
         </is>
       </c>
-      <c r="C6" s="60" t="n">
+      <c r="C6" s="61" t="n">
         <v>8500</v>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="56" t="n">
+      <c r="E6" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="56" t="n">
+      <c r="F6" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="56" t="n">
+      <c r="G6" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="56" t="n">
+      <c r="H6" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I6" s="48">
@@ -1929,27 +1988,27 @@
           <t>Suporte + capacitação</t>
         </is>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>Enfermeira ou licenciada: atende por telefone/WhatsApp, cria usuários e vai aos centros capacitar.</t>
         </is>
       </c>
-      <c r="C7" s="60" t="n">
+      <c r="C7" s="61" t="n">
         <v>5500</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="56" t="n">
+      <c r="E7" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="56" t="n">
+      <c r="F7" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="56" t="n">
+      <c r="G7" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="56" t="n">
+      <c r="H7" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I7" s="48">
@@ -1975,27 +2034,27 @@
           <t>Mesa de ajuda</t>
         </is>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Só atendimento remoto (telefone, WhatsApp, e-mail).</t>
         </is>
       </c>
-      <c r="C8" s="60" t="n">
+      <c r="C8" s="61" t="n">
         <v>4000</v>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="56" t="n">
+      <c r="E8" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="56" t="n">
+      <c r="F8" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="56" t="n">
+      <c r="G8" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="56" t="n">
+      <c r="H8" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I8" s="48">
@@ -2021,27 +2080,27 @@
           <t>Implantador / capacitador</t>
         </is>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>Vai a cada centro e hospital; 1 pessoa dá conta de ~40 centros por semestre de implantação.</t>
         </is>
       </c>
-      <c r="C9" s="60" t="n">
+      <c r="C9" s="61" t="n">
         <v>6000</v>
       </c>
-      <c r="D9" s="30" t="n">
+      <c r="D9" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="56" t="n">
+      <c r="E9" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="56" t="n">
+      <c r="F9" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="56" t="n">
+      <c r="G9" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="56" t="n">
+      <c r="H9" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I9" s="48">
@@ -2067,27 +2126,27 @@
           <t>Administrativo e financeiro (meio período)</t>
         </is>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Faturas ao município, cobranças, pagamentos.</t>
         </is>
       </c>
-      <c r="C10" s="60" t="n">
+      <c r="C10" s="61" t="n">
         <v>2500</v>
       </c>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="56" t="n">
+      <c r="E10" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="56" t="n">
+      <c r="F10" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="56" t="n">
+      <c r="G10" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="56" t="n">
+      <c r="H10" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I10" s="48">
@@ -2113,27 +2172,27 @@
           <t>Contador (externo)</t>
         </is>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="29" t="inlineStr">
         <is>
           <t>Impostos, balanços, folha de pagamento.</t>
         </is>
       </c>
-      <c r="C11" s="60" t="n">
+      <c r="C11" s="61" t="n">
         <v>1500</v>
       </c>
-      <c r="D11" s="30" t="n">
+      <c r="D11" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="56" t="n">
+      <c r="E11" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="56" t="n">
+      <c r="F11" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="56" t="n">
+      <c r="G11" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="56" t="n">
+      <c r="H11" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I11" s="48">
@@ -2159,27 +2218,27 @@
           <t>Advogado (externo, por demanda)</t>
         </is>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>Contratos, SENAPI, proteção de dados.</t>
         </is>
       </c>
-      <c r="C12" s="60" t="n">
+      <c r="C12" s="61" t="n">
         <v>1000</v>
       </c>
-      <c r="D12" s="30" t="n">
+      <c r="D12" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="56" t="n">
+      <c r="E12" s="57" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="56" t="n">
+      <c r="F12" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="56" t="n">
+      <c r="G12" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="56" t="n">
+      <c r="H12" s="57" t="n">
         <v>1</v>
       </c>
       <c r="I12" s="48">
@@ -2205,19 +2264,19 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E13" s="58">
+      <c r="E13" s="59">
         <f>SUM(E5:E12)</f>
         <v/>
       </c>
-      <c r="F13" s="58">
+      <c r="F13" s="59">
         <f>SUM(F5:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="58">
+      <c r="G13" s="59">
         <f>SUM(G5:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="58">
+      <c r="H13" s="59">
         <f>SUM(H5:H12)</f>
         <v/>
       </c>
@@ -2244,19 +2303,19 @@
           <t>Só pessoas contratadas (sem externos)</t>
         </is>
       </c>
-      <c r="E14" s="61">
+      <c r="E14" s="62">
         <f>SUMPRODUCT(E5:E12,1-$D$5:$D$12)</f>
         <v/>
       </c>
-      <c r="F14" s="61">
+      <c r="F14" s="62">
         <f>SUMPRODUCT(F5:F12,1-$D$5:$D$12)</f>
         <v/>
       </c>
-      <c r="G14" s="61">
+      <c r="G14" s="62">
         <f>SUMPRODUCT(G5:G12,1-$D$5:$D$12)</f>
         <v/>
       </c>
-      <c r="H14" s="61">
+      <c r="H14" s="62">
         <f>SUMPRODUCT(H5:H12,1-$D$5:$D$12)</f>
         <v/>
       </c>
@@ -2365,16 +2424,16 @@
           <t>Aluguel de sala (30–40 m²)</t>
         </is>
       </c>
-      <c r="B5" s="62" t="n">
+      <c r="B5" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="62" t="n">
+      <c r="C5" s="63" t="n">
         <v>2100</v>
       </c>
-      <c r="D5" s="62" t="n">
+      <c r="D5" s="63" t="n">
         <v>2800</v>
       </c>
-      <c r="E5" s="62" t="n">
+      <c r="E5" s="63" t="n">
         <v>2800</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2389,16 +2448,16 @@
           <t>Luz, internet e condomínio</t>
         </is>
       </c>
-      <c r="B6" s="62" t="n">
+      <c r="B6" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="62" t="n">
+      <c r="C6" s="63" t="n">
         <v>600</v>
       </c>
-      <c r="D6" s="62" t="n">
+      <c r="D6" s="63" t="n">
         <v>700</v>
       </c>
-      <c r="E6" s="62" t="n">
+      <c r="E6" s="63" t="n">
         <v>700</v>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
@@ -2409,16 +2468,16 @@
           <t>Transporte na cidade</t>
         </is>
       </c>
-      <c r="B7" s="62" t="n">
+      <c r="B7" s="63" t="n">
         <v>500</v>
       </c>
-      <c r="C7" s="62" t="n">
+      <c r="C7" s="63" t="n">
         <v>1200</v>
       </c>
-      <c r="D7" s="62" t="n">
+      <c r="D7" s="63" t="n">
         <v>1500</v>
       </c>
-      <c r="E7" s="62" t="n">
+      <c r="E7" s="63" t="n">
         <v>1500</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2433,16 +2492,16 @@
           <t>Viagens às províncias (passagem + diárias)</t>
         </is>
       </c>
-      <c r="B8" s="62" t="n">
+      <c r="B8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="62" t="n">
+      <c r="C8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="62" t="n">
+      <c r="D8" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="62" t="n">
+      <c r="E8" s="63" t="n">
         <v>4000</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2457,16 +2516,16 @@
           <t>Notebooks e celulares (divididos em 36 meses)</t>
         </is>
       </c>
-      <c r="B9" s="62" t="n">
+      <c r="B9" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="62" t="n">
+      <c r="C9" s="63" t="n">
         <v>700</v>
       </c>
-      <c r="D9" s="62" t="n">
+      <c r="D9" s="63" t="n">
         <v>1000</v>
       </c>
-      <c r="E9" s="62" t="n">
+      <c r="E9" s="63" t="n">
         <v>1000</v>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
@@ -2477,16 +2536,16 @@
           <t>Reserva para imprevistos</t>
         </is>
       </c>
-      <c r="B10" s="62" t="n">
+      <c r="B10" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="62" t="n">
+      <c r="C10" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="D10" s="62" t="n">
+      <c r="D10" s="63" t="n">
         <v>2000</v>
       </c>
-      <c r="E10" s="62" t="n">
+      <c r="E10" s="63" t="n">
         <v>3500</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2807,7 +2866,7 @@
           <t>TOTAL (US$/mês)</t>
         </is>
       </c>
-      <c r="D14" s="63">
+      <c r="D14" s="64">
         <f>SUM(D5:D13)</f>
         <v/>
       </c>
@@ -2891,7 +2950,7 @@
           <t>Tomas de PAP/VPH por centro por ano</t>
         </is>
       </c>
-      <c r="B6" s="57" t="n">
+      <c r="B6" s="58" t="n">
         <v>300</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2906,7 +2965,7 @@
           <t>Tomas por ano no município</t>
         </is>
       </c>
-      <c r="B7" s="61">
+      <c r="B7" s="62">
         <f>B5*B6</f>
         <v/>
       </c>
@@ -2918,7 +2977,7 @@
           <t>Folhas de papel por toma</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n">
+      <c r="B8" s="35" t="n">
         <v>3.5</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2933,7 +2992,7 @@
           <t>Custo por folha (papel + impressão/fotocópia, Bs)</t>
         </is>
       </c>
-      <c r="B9" s="35" t="n">
+      <c r="B9" s="36" t="n">
         <v>0.25</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2960,7 +3019,7 @@
           <t>Minutos de papelada economizados por toma</t>
         </is>
       </c>
-      <c r="B11" s="57" t="n">
+      <c r="B11" s="58" t="n">
         <v>15</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2975,7 +3034,7 @@
           <t>Horas por mês de informes do PAP por centro (SNIS, listas)</t>
         </is>
       </c>
-      <c r="B12" s="34" t="n">
+      <c r="B12" s="35" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2990,7 +3049,7 @@
           <t>Custo de uma hora de enfermeira/licenciada (Bs)</t>
         </is>
       </c>
-      <c r="B13" s="36">
+      <c r="B13" s="37">
         <f>6000/176*(1+Supostos!$B$15)</f>
         <v/>
       </c>
@@ -3006,7 +3065,7 @@
           <t>Horas devolvidas por ano</t>
         </is>
       </c>
-      <c r="B14" s="61">
+      <c r="B14" s="62">
         <f>B7*B11/60+B5*B12*12</f>
         <v/>
       </c>
@@ -3018,7 +3077,7 @@
           <t>Equivale a enfermeiras em tempo integral</t>
         </is>
       </c>
-      <c r="B15" s="37">
+      <c r="B15" s="38">
         <f>B14/(176*12)</f>
         <v/>
       </c>
@@ -3061,7 +3120,7 @@
           <t>Custo de repetir uma toma (Bs)</t>
         </is>
       </c>
-      <c r="B18" s="60" t="n">
+      <c r="B18" s="61" t="n">
         <v>60</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3083,16 +3142,16 @@
       <c r="C19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="38" t="inlineStr">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>ECONOMIA TOTAL POR ANO (Bs)</t>
         </is>
       </c>
-      <c r="B20" s="64">
+      <c r="B20" s="65">
         <f>B10+B16+B19</f>
         <v/>
       </c>
-      <c r="C20" s="40" t="inlineStr"/>
+      <c r="C20" s="41" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -3113,7 +3172,7 @@
         </is>
       </c>
       <c r="B22" s="46">
-        <f>Estabelecimentos!E12*12</f>
+        <f>Estabelecimentos!E13*12</f>
         <v/>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3225,7 +3284,7 @@
           <t>Lesões de alto grau detectadas por ano</t>
         </is>
       </c>
-      <c r="B7" s="61">
+      <c r="B7" s="62">
         <f>B5*B6</f>
         <v/>
       </c>
@@ -3267,7 +3326,7 @@
           <t>Mulheres a mais tratadas a tempo, por ano</t>
         </is>
       </c>
-      <c r="B10" s="61">
+      <c r="B10" s="62">
         <f>B7*(B9-B8)</f>
         <v/>
       </c>
@@ -3294,7 +3353,7 @@
           <t>Cânceres evitados por ano</t>
         </is>
       </c>
-      <c r="B12" s="37">
+      <c r="B12" s="38">
         <f>B10*B11</f>
         <v/>
       </c>
@@ -3322,11 +3381,11 @@
           <t>VIDAS SALVAS POR ANO</t>
         </is>
       </c>
-      <c r="B14" s="41">
+      <c r="B14" s="42">
         <f>B12*B13</f>
         <v/>
       </c>
-      <c r="C14" s="40" t="inlineStr"/>
+      <c r="C14" s="41" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -3334,7 +3393,7 @@
           <t>Filhos por mãe que morre de câncer de colo</t>
         </is>
       </c>
-      <c r="B15" s="34" t="n">
+      <c r="B15" s="35" t="n">
         <v>2.1</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3349,11 +3408,11 @@
           <t>CRIANÇAS QUE NÃO FICAM ÓRFÃS POR ANO</t>
         </is>
       </c>
-      <c r="B16" s="41">
+      <c r="B16" s="42">
         <f>B14*B15</f>
         <v/>
       </c>
-      <c r="C16" s="40" t="inlineStr"/>
+      <c r="C16" s="41" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3361,7 +3420,7 @@
           <t>Anos de vida perdidos por cada morte</t>
         </is>
       </c>
-      <c r="B17" s="57" t="n">
+      <c r="B17" s="58" t="n">
         <v>20</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3376,7 +3435,7 @@
           <t>Anos de vida salvos por ano</t>
         </is>
       </c>
-      <c r="B18" s="61">
+      <c r="B18" s="62">
         <f>B14*B17</f>
         <v/>
       </c>
@@ -3388,7 +3447,7 @@
           <t>Renda nacional por habitante (US$/ano)</t>
         </is>
       </c>
-      <c r="B19" s="65" t="n">
+      <c r="B19" s="56" t="n">
         <v>3690</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3419,7 +3478,7 @@
           <t>Valor estatístico de uma vida na Bolívia (US$)</t>
         </is>
       </c>
-      <c r="B21" s="65" t="n">
+      <c r="B21" s="56" t="n">
         <v>127000</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3446,7 +3505,7 @@
           <t>Custo para o SUS de tratar um câncer de colo (Bs)</t>
         </is>
       </c>
-      <c r="B23" s="60" t="n">
+      <c r="B23" s="61" t="n">
         <v>60000</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3461,7 +3520,7 @@
           <t>Custo de tratar uma lesão de alto grau a tempo (Bs)</t>
         </is>
       </c>
-      <c r="B24" s="60" t="n">
+      <c r="B24" s="61" t="n">
         <v>800</v>
       </c>
       <c r="C24" s="2" t="inlineStr">

</xml_diff>